<commit_message>
update item with metafield, burger pos range, publish menu
</commit_message>
<xml_diff>
--- a/Data/Item_log_Template.xlsx
+++ b/Data/Item_log_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MKR7550\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MKR7550\Documents\UiPath\RE_CFCAutomation\RE_CFCAutomation\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE3F012C-E2CC-4060-BB76-BA15C1BD45D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{616B7CC5-29FA-4A24-A3AF-E09230EBDEC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{3203513D-5511-4B48-8E59-55BB4D7708A1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Action</t>
   </si>
@@ -57,6 +57,15 @@
   </si>
   <si>
     <t>API_Status_Code</t>
+  </si>
+  <si>
+    <t>Product Code</t>
+  </si>
+  <si>
+    <t>Variant Code</t>
+  </si>
+  <si>
+    <t>Item Type</t>
   </si>
 </sst>
 </file>
@@ -459,42 +468,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10DE1B90-BA82-4B98-9093-0B8DADE7BBCD}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="17" style="2" customWidth="1"/>
-    <col min="3" max="3" width="28.42578125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="12" style="2" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="76.140625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="14.28515625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="17" style="2" customWidth="1"/>
+    <col min="6" max="6" width="28.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="12" style="2" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="76.140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>